<commit_message>
Update with new Pgt representatives
</commit_message>
<xml_diff>
--- a/resources/pgt/pgt_sample_metadata.xlsx
+++ b/resources/pgt/pgt_sample_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vof23jop/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MARPLE_MayUpdate/resources/pgt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBE575A-DD8B-594A-9072-8DA204571B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E2614ED-8754-EC4C-BA9A-88E28BA742E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-1460" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36000" yWindow="-1360" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">metadata!$A$1:$S$1</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1844" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1876" uniqueCount="466">
   <si>
     <t>accession</t>
   </si>
@@ -1401,6 +1401,42 @@
   </si>
   <si>
     <t>#E7DCAE</t>
+  </si>
+  <si>
+    <t>NewRepIsol_barcode02</t>
+  </si>
+  <si>
+    <t>DK263_21</t>
+  </si>
+  <si>
+    <t>13GER06_1</t>
+  </si>
+  <si>
+    <t>DK177b1_24</t>
+  </si>
+  <si>
+    <t>IT100a_17</t>
+  </si>
+  <si>
+    <t>UA49_24</t>
+  </si>
+  <si>
+    <t>NULL (Clade IV-C)</t>
+  </si>
+  <si>
+    <t>13GER06 (Clade IV-C)</t>
+  </si>
+  <si>
+    <t>DK263 (Clade IV-B)</t>
+  </si>
+  <si>
+    <t>DK177b1 (Clade IV-F)</t>
+  </si>
+  <si>
+    <t>IT100a (Clade III-B)</t>
+  </si>
+  <si>
+    <t>UA49 (Clade IV-C)</t>
   </si>
 </sst>
 </file>
@@ -1734,7 +1770,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1807,8 +1843,7 @@
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyFill="1"/>
@@ -1827,847 +1862,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="96">
-    <dxf>
-      <font>
-        <color rgb="FF2C3B49"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF8BB4DA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4F5C66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB3CFE5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4E55"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E0F1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF58452F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDBA7E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4C2815"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD57039"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF46301A"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE69E56"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF42503E"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB5D8A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF495146"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E7C8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E351F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF61AB64"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF30422C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF94C986"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4739"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7DCAE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF544443"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE0B6B3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF2C3B49"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF8BB4DA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4F5C66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB3CFE5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4E55"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E0F1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF58452F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDBA7E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4C2815"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD57039"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF46301A"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE69E56"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF42503E"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB5D8A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF495146"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E7C8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E351F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF61AB64"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF30422C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF94C986"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4739"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7DCAE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF544443"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE0B6B3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF2C3B49"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF8BB4DA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4F5C66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB3CFE5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4E55"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E0F1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF58452F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDBA7E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4C2815"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD57039"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF46301A"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE69E56"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF42503E"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB5D8A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF495146"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E7C8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E351F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF61AB64"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF30422C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF94C986"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4739"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7DCAE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF544443"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE0B6B3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF2C3B49"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF8BB4DA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4F5C66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB3CFE5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4E55"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E0F1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF58452F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDBA7E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4C2815"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD57039"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF46301A"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE69E56"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF42503E"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB5D8A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF495146"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E7C8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E351F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF61AB64"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF30422C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF94C986"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4739"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7DCAE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF544443"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE0B6B3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF2C3B49"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF8BB4DA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4F5C66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB3CFE5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4E55"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E0F1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF58452F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDBA7E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4C2815"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD57039"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF46301A"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE69E56"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF42503E"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB5D8A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF495146"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E7C8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E351F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF61AB64"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF30422C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF94C986"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4739"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7DCAE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF544443"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE0B6B3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF2C3B49"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF8BB4DA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4F5C66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB3CFE5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4E55"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E0F1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF58452F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDBA7E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4C2815"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD57039"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF46301A"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE69E56"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF42503E"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB5D8A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF495146"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E7C8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E351F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF61AB64"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF30422C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF94C986"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4739"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7DCAE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF544443"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE0B6B3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF2C3B49"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF8BB4DA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4F5C66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB3CFE5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4E55"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E0F1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF58452F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEDBA7E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4C2815"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD57039"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF46301A"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE69E56"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF42503E"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB5D8A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF495146"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD3E7C8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E351F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF61AB64"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF30422C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF94C986"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF4A4739"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7DCAE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF544443"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE0B6B3"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <font>
         <color rgb="FF2C3B49"/>
@@ -3102,7 +2297,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S107"/>
+  <dimension ref="A1:S113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="42" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
@@ -3139,7 +2334,7 @@
       <c r="D1" t="s">
         <v>296</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" t="s">
         <v>328</v>
       </c>
       <c r="F1" s="4" t="s">
@@ -3198,7 +2393,7 @@
       <c r="D2" t="s">
         <v>297</v>
       </c>
-      <c r="E2" s="35" t="s">
+      <c r="E2" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F2" t="s">
@@ -3257,7 +2452,7 @@
       <c r="D3" t="s">
         <v>297</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="E3" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F3" t="s">
@@ -3316,7 +2511,7 @@
       <c r="D4" t="s">
         <v>297</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="E4" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F4" t="s">
@@ -3375,7 +2570,7 @@
       <c r="D5" t="s">
         <v>297</v>
       </c>
-      <c r="E5" s="35" t="s">
+      <c r="E5" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F5" t="s">
@@ -3434,7 +2629,7 @@
       <c r="D6" t="s">
         <v>297</v>
       </c>
-      <c r="E6" s="35" t="s">
+      <c r="E6" s="34" t="s">
         <v>330</v>
       </c>
       <c r="F6" t="s">
@@ -3493,7 +2688,7 @@
       <c r="D7" t="s">
         <v>297</v>
       </c>
-      <c r="E7" s="35" t="s">
+      <c r="E7" s="34" t="s">
         <v>330</v>
       </c>
       <c r="F7" t="s">
@@ -3552,7 +2747,7 @@
       <c r="D8" t="s">
         <v>299</v>
       </c>
-      <c r="E8" s="35" t="s">
+      <c r="E8" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F8" t="s">
@@ -3611,7 +2806,7 @@
       <c r="D9" t="s">
         <v>299</v>
       </c>
-      <c r="E9" s="35" t="s">
+      <c r="E9" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F9" t="s">
@@ -3670,7 +2865,7 @@
       <c r="D10" t="s">
         <v>299</v>
       </c>
-      <c r="E10" s="35" t="s">
+      <c r="E10" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F10" t="s">
@@ -3729,7 +2924,7 @@
       <c r="D11" t="s">
         <v>299</v>
       </c>
-      <c r="E11" s="35" t="s">
+      <c r="E11" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F11" t="s">
@@ -3788,7 +2983,7 @@
       <c r="D12" t="s">
         <v>300</v>
       </c>
-      <c r="E12" s="35" t="s">
+      <c r="E12" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F12" t="s">
@@ -3847,7 +3042,7 @@
       <c r="D13" t="s">
         <v>300</v>
       </c>
-      <c r="E13" s="35" t="s">
+      <c r="E13" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F13" t="s">
@@ -3906,7 +3101,7 @@
       <c r="D14" t="s">
         <v>300</v>
       </c>
-      <c r="E14" s="35" t="s">
+      <c r="E14" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F14" t="s">
@@ -3965,7 +3160,7 @@
       <c r="D15" t="s">
         <v>300</v>
       </c>
-      <c r="E15" s="35" t="s">
+      <c r="E15" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F15" t="s">
@@ -4024,7 +3219,7 @@
       <c r="D16" t="s">
         <v>300</v>
       </c>
-      <c r="E16" s="35" t="s">
+      <c r="E16" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F16" t="s">
@@ -4083,7 +3278,7 @@
       <c r="D17" t="s">
         <v>300</v>
       </c>
-      <c r="E17" s="35" t="s">
+      <c r="E17" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F17" t="s">
@@ -4142,7 +3337,7 @@
       <c r="D18" t="s">
         <v>300</v>
       </c>
-      <c r="E18" s="35" t="s">
+      <c r="E18" s="34" t="s">
         <v>337</v>
       </c>
       <c r="F18" t="s">
@@ -4201,7 +3396,7 @@
       <c r="D19" t="s">
         <v>300</v>
       </c>
-      <c r="E19" s="35" t="s">
+      <c r="E19" s="34" t="s">
         <v>337</v>
       </c>
       <c r="F19" t="s">
@@ -4260,7 +3455,7 @@
       <c r="D20" t="s">
         <v>342</v>
       </c>
-      <c r="E20" s="35" t="s">
+      <c r="E20" s="34" t="s">
         <v>340</v>
       </c>
       <c r="F20" t="s">
@@ -4319,7 +3514,7 @@
       <c r="D21" t="s">
         <v>297</v>
       </c>
-      <c r="E21" s="35" t="s">
+      <c r="E21" s="34" t="s">
         <v>334</v>
       </c>
       <c r="F21" t="s">
@@ -4378,7 +3573,7 @@
       <c r="D22" t="s">
         <v>299</v>
       </c>
-      <c r="E22" s="35" t="s">
+      <c r="E22" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F22" t="s">
@@ -4437,7 +3632,7 @@
       <c r="D23" t="s">
         <v>299</v>
       </c>
-      <c r="E23" s="35" t="s">
+      <c r="E23" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F23" t="s">
@@ -4496,7 +3691,7 @@
       <c r="D24" t="s">
         <v>299</v>
       </c>
-      <c r="E24" s="35" t="s">
+      <c r="E24" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F24" t="s">
@@ -4555,7 +3750,7 @@
       <c r="D25" t="s">
         <v>299</v>
       </c>
-      <c r="E25" s="35" t="s">
+      <c r="E25" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F25" t="s">
@@ -4614,7 +3809,7 @@
       <c r="D26" t="s">
         <v>299</v>
       </c>
-      <c r="E26" s="35" t="s">
+      <c r="E26" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F26" t="s">
@@ -4673,7 +3868,7 @@
       <c r="D27" t="s">
         <v>299</v>
       </c>
-      <c r="E27" s="35" t="s">
+      <c r="E27" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F27" t="s">
@@ -4732,7 +3927,7 @@
       <c r="D28" t="s">
         <v>299</v>
       </c>
-      <c r="E28" s="35" t="s">
+      <c r="E28" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F28" t="s">
@@ -4791,7 +3986,7 @@
       <c r="D29" t="s">
         <v>301</v>
       </c>
-      <c r="E29" s="35" t="s">
+      <c r="E29" s="34" t="s">
         <v>340</v>
       </c>
       <c r="F29" t="s">
@@ -4850,7 +4045,7 @@
       <c r="D30" t="s">
         <v>301</v>
       </c>
-      <c r="E30" s="35" t="s">
+      <c r="E30" s="34" t="s">
         <v>340</v>
       </c>
       <c r="F30" t="s">
@@ -4909,7 +4104,7 @@
       <c r="D31" t="s">
         <v>297</v>
       </c>
-      <c r="E31" s="35" t="s">
+      <c r="E31" s="34" t="s">
         <v>336</v>
       </c>
       <c r="F31" t="s">
@@ -4968,7 +4163,7 @@
       <c r="D32" t="s">
         <v>297</v>
       </c>
-      <c r="E32" s="35" t="s">
+      <c r="E32" s="34" t="s">
         <v>336</v>
       </c>
       <c r="F32" t="s">
@@ -5027,7 +4222,7 @@
       <c r="D33" t="s">
         <v>297</v>
       </c>
-      <c r="E33" s="35" t="s">
+      <c r="E33" s="34" t="s">
         <v>336</v>
       </c>
       <c r="F33" t="s">
@@ -5086,7 +4281,7 @@
       <c r="D34" t="s">
         <v>297</v>
       </c>
-      <c r="E34" s="35" t="s">
+      <c r="E34" s="34" t="s">
         <v>336</v>
       </c>
       <c r="F34" t="s">
@@ -5145,7 +4340,7 @@
       <c r="D35" t="s">
         <v>297</v>
       </c>
-      <c r="E35" s="35" t="s">
+      <c r="E35" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F35" t="s">
@@ -5204,7 +4399,7 @@
       <c r="D36" t="s">
         <v>342</v>
       </c>
-      <c r="E36" s="35" t="s">
+      <c r="E36" s="34" t="s">
         <v>332</v>
       </c>
       <c r="F36" t="s">
@@ -5263,7 +4458,7 @@
       <c r="D37" t="s">
         <v>297</v>
       </c>
-      <c r="E37" s="35" t="s">
+      <c r="E37" s="34" t="s">
         <v>103</v>
       </c>
       <c r="F37" t="s">
@@ -5310,7 +4505,7 @@
       <c r="D38" t="s">
         <v>297</v>
       </c>
-      <c r="E38" s="35" t="s">
+      <c r="E38" s="34" t="s">
         <v>103</v>
       </c>
       <c r="F38" t="s">
@@ -5357,7 +4552,7 @@
       <c r="D39" t="s">
         <v>299</v>
       </c>
-      <c r="E39" s="35" t="s">
+      <c r="E39" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F39" t="s">
@@ -5414,7 +4609,7 @@
       <c r="D40" t="s">
         <v>299</v>
       </c>
-      <c r="E40" s="35" t="s">
+      <c r="E40" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F40" t="s">
@@ -5471,7 +4666,7 @@
       <c r="D41" t="s">
         <v>299</v>
       </c>
-      <c r="E41" s="35" t="s">
+      <c r="E41" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F41" t="s">
@@ -5528,7 +4723,7 @@
       <c r="D42" t="s">
         <v>299</v>
       </c>
-      <c r="E42" s="35" t="s">
+      <c r="E42" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F42" t="s">
@@ -5584,7 +4779,7 @@
       <c r="D43" t="s">
         <v>299</v>
       </c>
-      <c r="E43" s="35" t="s">
+      <c r="E43" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F43" t="s">
@@ -5640,7 +4835,7 @@
       <c r="D44" t="s">
         <v>299</v>
       </c>
-      <c r="E44" s="35" t="s">
+      <c r="E44" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F44" t="s">
@@ -5697,7 +4892,7 @@
       <c r="D45" t="s">
         <v>299</v>
       </c>
-      <c r="E45" s="35" t="s">
+      <c r="E45" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F45" t="s">
@@ -5754,14 +4949,14 @@
       <c r="D46" t="s">
         <v>299</v>
       </c>
-      <c r="E46" s="35" t="s">
+      <c r="E46" s="34" t="s">
         <v>332</v>
       </c>
       <c r="F46" t="s">
         <v>59</v>
       </c>
       <c r="G46" s="5" t="str">
-        <f>_xlfn.CONCAT("19", LEFT(B46,2))</f>
+        <f t="shared" ref="G46:G53" si="0">_xlfn.CONCAT("19", LEFT(B46,2))</f>
         <v>1996</v>
       </c>
       <c r="H46">
@@ -5811,14 +5006,14 @@
       <c r="D47" t="s">
         <v>299</v>
       </c>
-      <c r="E47" s="35" t="s">
+      <c r="E47" s="34" t="s">
         <v>330</v>
       </c>
       <c r="F47" t="s">
         <v>60</v>
       </c>
       <c r="G47" s="5" t="str">
-        <f>_xlfn.CONCAT("19", LEFT(B47,2))</f>
+        <f t="shared" si="0"/>
         <v>1983</v>
       </c>
       <c r="H47">
@@ -5868,14 +5063,14 @@
       <c r="D48" t="s">
         <v>299</v>
       </c>
-      <c r="E48" s="35" t="s">
+      <c r="E48" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F48" t="s">
         <v>61</v>
       </c>
       <c r="G48" s="5" t="str">
-        <f>_xlfn.CONCAT("19", LEFT(B48,2))</f>
+        <f t="shared" si="0"/>
         <v>1987</v>
       </c>
       <c r="H48">
@@ -5925,14 +5120,14 @@
       <c r="D49" t="s">
         <v>299</v>
       </c>
-      <c r="E49" s="35" t="s">
+      <c r="E49" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F49" t="s">
         <v>62</v>
       </c>
       <c r="G49" s="5" t="str">
-        <f>_xlfn.CONCAT("19", LEFT(B49,2))</f>
+        <f t="shared" si="0"/>
         <v>1983</v>
       </c>
       <c r="H49">
@@ -5982,14 +5177,14 @@
       <c r="D50" t="s">
         <v>299</v>
       </c>
-      <c r="E50" s="35" t="s">
+      <c r="E50" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F50" t="s">
         <v>63</v>
       </c>
       <c r="G50" s="5" t="str">
-        <f>_xlfn.CONCAT("19", LEFT(B50,2))</f>
+        <f t="shared" si="0"/>
         <v>1985</v>
       </c>
       <c r="H50">
@@ -6039,14 +5234,14 @@
       <c r="D51" t="s">
         <v>299</v>
       </c>
-      <c r="E51" s="35" t="s">
+      <c r="E51" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F51" t="s">
         <v>64</v>
       </c>
       <c r="G51" s="5" t="str">
-        <f>_xlfn.CONCAT("19", LEFT(B51,2))</f>
+        <f t="shared" si="0"/>
         <v>1980</v>
       </c>
       <c r="H51">
@@ -6096,14 +5291,14 @@
       <c r="D52" t="s">
         <v>300</v>
       </c>
-      <c r="E52" s="35" t="s">
+      <c r="E52" s="34" t="s">
         <v>337</v>
       </c>
       <c r="F52" t="s">
         <v>65</v>
       </c>
       <c r="G52" s="5" t="str">
-        <f>_xlfn.CONCAT("19", LEFT(B52,2))</f>
+        <f t="shared" si="0"/>
         <v>1986</v>
       </c>
       <c r="H52">
@@ -6153,14 +5348,14 @@
       <c r="D53" t="s">
         <v>297</v>
       </c>
-      <c r="E53" s="35" t="s">
+      <c r="E53" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F53" t="s">
         <v>66</v>
       </c>
       <c r="G53" s="5" t="str">
-        <f>_xlfn.CONCAT("19", LEFT(B53,2))</f>
+        <f t="shared" si="0"/>
         <v>1986</v>
       </c>
       <c r="H53">
@@ -6210,7 +5405,7 @@
       <c r="D54" t="s">
         <v>299</v>
       </c>
-      <c r="E54" s="35" t="s">
+      <c r="E54" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F54" t="s">
@@ -6267,7 +5462,7 @@
       <c r="D55" t="s">
         <v>300</v>
       </c>
-      <c r="E55" s="35" t="s">
+      <c r="E55" s="34" t="s">
         <v>333</v>
       </c>
       <c r="F55" t="s">
@@ -6324,7 +5519,7 @@
       <c r="D56" t="s">
         <v>299</v>
       </c>
-      <c r="E56" s="35" t="s">
+      <c r="E56" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F56" t="s">
@@ -6381,7 +5576,7 @@
       <c r="D57" t="s">
         <v>297</v>
       </c>
-      <c r="E57" s="35" t="s">
+      <c r="E57" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F57" t="s">
@@ -6438,7 +5633,7 @@
       <c r="D58" t="s">
         <v>299</v>
       </c>
-      <c r="E58" s="35" t="s">
+      <c r="E58" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F58" t="s">
@@ -6495,7 +5690,7 @@
       <c r="D59" t="s">
         <v>300</v>
       </c>
-      <c r="E59" s="35" t="s">
+      <c r="E59" s="34" t="s">
         <v>336</v>
       </c>
       <c r="F59" t="s">
@@ -6551,7 +5746,7 @@
       <c r="D60" t="s">
         <v>300</v>
       </c>
-      <c r="E60" s="35" t="s">
+      <c r="E60" s="34" t="s">
         <v>336</v>
       </c>
       <c r="F60" t="s">
@@ -6607,7 +5802,7 @@
       <c r="D61" t="s">
         <v>299</v>
       </c>
-      <c r="E61" s="35" t="s">
+      <c r="E61" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F61" t="s">
@@ -6664,7 +5859,7 @@
       <c r="D62" t="s">
         <v>299</v>
       </c>
-      <c r="E62" s="35" t="s">
+      <c r="E62" s="34" t="s">
         <v>333</v>
       </c>
       <c r="F62" t="s">
@@ -6721,7 +5916,7 @@
       <c r="D63" t="s">
         <v>297</v>
       </c>
-      <c r="E63" s="35" t="s">
+      <c r="E63" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F63" t="s">
@@ -6778,7 +5973,7 @@
       <c r="D64" t="s">
         <v>299</v>
       </c>
-      <c r="E64" s="35" t="s">
+      <c r="E64" s="34" t="s">
         <v>333</v>
       </c>
       <c r="F64" t="s">
@@ -6835,7 +6030,7 @@
       <c r="D65" t="s">
         <v>342</v>
       </c>
-      <c r="E65" s="35" t="s">
+      <c r="E65" s="34" t="s">
         <v>332</v>
       </c>
       <c r="F65" t="s">
@@ -6892,7 +6087,7 @@
       <c r="D66" t="s">
         <v>342</v>
       </c>
-      <c r="E66" s="35" t="s">
+      <c r="E66" s="34" t="s">
         <v>332</v>
       </c>
       <c r="F66" t="s">
@@ -6949,7 +6144,7 @@
       <c r="D67" t="s">
         <v>342</v>
       </c>
-      <c r="E67" s="35" t="s">
+      <c r="E67" s="34" t="s">
         <v>335</v>
       </c>
       <c r="F67" t="s">
@@ -7006,7 +6201,7 @@
       <c r="D68" t="s">
         <v>342</v>
       </c>
-      <c r="E68" s="35" t="s">
+      <c r="E68" s="34" t="s">
         <v>340</v>
       </c>
       <c r="F68" t="s">
@@ -7063,7 +6258,7 @@
       <c r="D69" t="s">
         <v>342</v>
       </c>
-      <c r="E69" s="35" t="s">
+      <c r="E69" s="34" t="s">
         <v>340</v>
       </c>
       <c r="F69" t="s">
@@ -7120,7 +6315,7 @@
       <c r="D70" t="s">
         <v>342</v>
       </c>
-      <c r="E70" s="35" t="s">
+      <c r="E70" s="34" t="s">
         <v>335</v>
       </c>
       <c r="F70" t="s">
@@ -7177,7 +6372,7 @@
       <c r="D71" t="s">
         <v>342</v>
       </c>
-      <c r="E71" s="35" t="s">
+      <c r="E71" s="34" t="s">
         <v>340</v>
       </c>
       <c r="F71" t="s">
@@ -7234,7 +6429,7 @@
       <c r="D72" t="s">
         <v>342</v>
       </c>
-      <c r="E72" s="35" t="s">
+      <c r="E72" s="34" t="s">
         <v>332</v>
       </c>
       <c r="F72" t="s">
@@ -7291,7 +6486,7 @@
       <c r="D73" t="s">
         <v>342</v>
       </c>
-      <c r="E73" s="35" t="s">
+      <c r="E73" s="34" t="s">
         <v>332</v>
       </c>
       <c r="F73" t="s">
@@ -7348,7 +6543,7 @@
       <c r="D74" t="s">
         <v>342</v>
       </c>
-      <c r="E74" s="35" t="s">
+      <c r="E74" s="34" t="s">
         <v>340</v>
       </c>
       <c r="F74" t="s">
@@ -7405,7 +6600,7 @@
       <c r="D75" t="s">
         <v>342</v>
       </c>
-      <c r="E75" s="35" t="s">
+      <c r="E75" s="34" t="s">
         <v>335</v>
       </c>
       <c r="F75" t="s">
@@ -7462,7 +6657,7 @@
       <c r="D76" t="s">
         <v>298</v>
       </c>
-      <c r="E76" s="35" t="s">
+      <c r="E76" s="34" t="s">
         <v>332</v>
       </c>
       <c r="F76" t="s">
@@ -7521,7 +6716,7 @@
       <c r="D77" t="s">
         <v>299</v>
       </c>
-      <c r="E77" s="35" t="s">
+      <c r="E77" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F77" t="s">
@@ -7574,7 +6769,7 @@
       <c r="D78" t="s">
         <v>299</v>
       </c>
-      <c r="E78" s="35" t="s">
+      <c r="E78" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F78" t="s">
@@ -7627,7 +6822,7 @@
       <c r="D79" t="s">
         <v>299</v>
       </c>
-      <c r="E79" s="35" t="s">
+      <c r="E79" s="34" t="s">
         <v>337</v>
       </c>
       <c r="F79" t="s">
@@ -7680,7 +6875,7 @@
       <c r="D80" t="s">
         <v>299</v>
       </c>
-      <c r="E80" s="35" t="s">
+      <c r="E80" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F80" t="s">
@@ -7733,7 +6928,7 @@
       <c r="D81" t="s">
         <v>299</v>
       </c>
-      <c r="E81" s="35" t="s">
+      <c r="E81" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F81" t="s">
@@ -7786,7 +6981,7 @@
       <c r="D82" t="s">
         <v>300</v>
       </c>
-      <c r="E82" s="35" t="s">
+      <c r="E82" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F82" t="s">
@@ -7839,7 +7034,7 @@
       <c r="D83" t="s">
         <v>299</v>
       </c>
-      <c r="E83" s="35" t="s">
+      <c r="E83" s="34" t="s">
         <v>337</v>
       </c>
       <c r="F83" t="s">
@@ -7892,7 +7087,7 @@
       <c r="D84" t="s">
         <v>299</v>
       </c>
-      <c r="E84" s="35" t="s">
+      <c r="E84" s="34" t="s">
         <v>339</v>
       </c>
       <c r="F84" t="s">
@@ -7945,7 +7140,7 @@
       <c r="D85" t="s">
         <v>301</v>
       </c>
-      <c r="E85" s="35" t="s">
+      <c r="E85" s="34" t="s">
         <v>335</v>
       </c>
       <c r="F85" t="s">
@@ -7998,7 +7193,7 @@
       <c r="D86" t="s">
         <v>342</v>
       </c>
-      <c r="E86" s="35" t="s">
+      <c r="E86" s="34" t="s">
         <v>332</v>
       </c>
       <c r="F86" t="s">
@@ -8051,7 +7246,7 @@
       <c r="D87" t="s">
         <v>342</v>
       </c>
-      <c r="E87" s="35" t="s">
+      <c r="E87" s="34" t="s">
         <v>340</v>
       </c>
       <c r="F87" t="s">
@@ -8104,7 +7299,7 @@
       <c r="D88" t="s">
         <v>342</v>
       </c>
-      <c r="E88" s="35" t="s">
+      <c r="E88" s="34" t="s">
         <v>332</v>
       </c>
       <c r="F88" t="s">
@@ -8157,7 +7352,7 @@
       <c r="D89" t="s">
         <v>342</v>
       </c>
-      <c r="E89" s="35" t="s">
+      <c r="E89" s="34" t="s">
         <v>340</v>
       </c>
       <c r="F89" t="s">
@@ -8210,7 +7405,7 @@
       <c r="D90" t="s">
         <v>342</v>
       </c>
-      <c r="E90" s="35" t="s">
+      <c r="E90" s="34" t="s">
         <v>335</v>
       </c>
       <c r="F90" t="s">
@@ -8263,7 +7458,7 @@
       <c r="D91" t="s">
         <v>297</v>
       </c>
-      <c r="E91" s="35" t="s">
+      <c r="E91" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F91" t="s">
@@ -8316,7 +7511,7 @@
       <c r="D92" t="s">
         <v>299</v>
       </c>
-      <c r="E92" s="35" t="s">
+      <c r="E92" s="34" t="s">
         <v>338</v>
       </c>
       <c r="F92" t="s">
@@ -8369,7 +7564,7 @@
       <c r="D93" t="s">
         <v>342</v>
       </c>
-      <c r="E93" s="35" t="s">
+      <c r="E93" s="34" t="s">
         <v>335</v>
       </c>
       <c r="F93" t="s">
@@ -8422,7 +7617,7 @@
       <c r="D94" t="s">
         <v>342</v>
       </c>
-      <c r="E94" s="35" t="s">
+      <c r="E94" s="34" t="s">
         <v>335</v>
       </c>
       <c r="F94" t="s">
@@ -8475,7 +7670,7 @@
       <c r="D95" t="s">
         <v>298</v>
       </c>
-      <c r="E95" s="35" t="s">
+      <c r="E95" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F95" t="s">
@@ -8534,7 +7729,7 @@
       <c r="D96" t="s">
         <v>298</v>
       </c>
-      <c r="E96" s="35" t="s">
+      <c r="E96" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F96" t="s">
@@ -8593,7 +7788,7 @@
       <c r="D97" t="s">
         <v>298</v>
       </c>
-      <c r="E97" s="35" t="s">
+      <c r="E97" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F97" t="s">
@@ -8652,7 +7847,7 @@
       <c r="D98" t="s">
         <v>298</v>
       </c>
-      <c r="E98" s="35" t="s">
+      <c r="E98" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F98" t="s">
@@ -8711,7 +7906,7 @@
       <c r="D99" t="s">
         <v>298</v>
       </c>
-      <c r="E99" s="35" t="s">
+      <c r="E99" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F99" t="s">
@@ -8770,7 +7965,7 @@
       <c r="D100" t="s">
         <v>298</v>
       </c>
-      <c r="E100" s="35" t="s">
+      <c r="E100" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F100" t="s">
@@ -8829,7 +8024,7 @@
       <c r="D101" t="s">
         <v>297</v>
       </c>
-      <c r="E101" s="35" t="s">
+      <c r="E101" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F101" t="s">
@@ -8888,7 +8083,7 @@
       <c r="D102" t="s">
         <v>299</v>
       </c>
-      <c r="E102" s="35" t="s">
+      <c r="E102" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F102" t="s">
@@ -8947,7 +8142,7 @@
       <c r="D103" t="s">
         <v>299</v>
       </c>
-      <c r="E103" s="35" t="s">
+      <c r="E103" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F103" t="s">
@@ -9006,7 +8201,7 @@
       <c r="D104" t="s">
         <v>299</v>
       </c>
-      <c r="E104" s="35" t="s">
+      <c r="E104" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F104" t="s">
@@ -9065,7 +8260,7 @@
       <c r="D105" t="s">
         <v>299</v>
       </c>
-      <c r="E105" s="35" t="s">
+      <c r="E105" s="34" t="s">
         <v>331</v>
       </c>
       <c r="F105" t="s">
@@ -9124,7 +8319,7 @@
       <c r="D106" t="s">
         <v>298</v>
       </c>
-      <c r="E106" s="35" t="s">
+      <c r="E106" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F106" t="s">
@@ -9183,7 +8378,7 @@
       <c r="D107" t="s">
         <v>298</v>
       </c>
-      <c r="E107" s="35" t="s">
+      <c r="E107" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F107" t="s">
@@ -9227,6 +8422,114 @@
       </c>
       <c r="S107">
         <v>0.97170362863935766</v>
+      </c>
+    </row>
+    <row r="108" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>454</v>
+      </c>
+      <c r="B108" t="s">
+        <v>460</v>
+      </c>
+      <c r="E108" s="34" t="s">
+        <v>336</v>
+      </c>
+      <c r="F108" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="109" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>455</v>
+      </c>
+      <c r="B109" t="s">
+        <v>462</v>
+      </c>
+      <c r="C109" t="s">
+        <v>254</v>
+      </c>
+      <c r="D109" t="s">
+        <v>297</v>
+      </c>
+      <c r="E109" s="34" t="s">
+        <v>338</v>
+      </c>
+      <c r="F109" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="110" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>456</v>
+      </c>
+      <c r="B110" t="s">
+        <v>461</v>
+      </c>
+      <c r="C110" t="s">
+        <v>407</v>
+      </c>
+      <c r="D110" t="s">
+        <v>297</v>
+      </c>
+      <c r="E110" s="34" t="s">
+        <v>338</v>
+      </c>
+      <c r="F110" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="111" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>457</v>
+      </c>
+      <c r="B111" t="s">
+        <v>463</v>
+      </c>
+      <c r="C111" t="s">
+        <v>254</v>
+      </c>
+      <c r="D111" t="s">
+        <v>297</v>
+      </c>
+      <c r="E111" s="34" t="s">
+        <v>338</v>
+      </c>
+      <c r="F111" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="112" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>458</v>
+      </c>
+      <c r="B112" t="s">
+        <v>464</v>
+      </c>
+      <c r="C112" t="s">
+        <v>261</v>
+      </c>
+      <c r="D112" t="s">
+        <v>297</v>
+      </c>
+      <c r="E112" s="34" t="s">
+        <v>336</v>
+      </c>
+      <c r="F112" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>459</v>
+      </c>
+      <c r="B113" t="s">
+        <v>465</v>
+      </c>
+      <c r="E113" s="34" t="s">
+        <v>338</v>
+      </c>
+      <c r="F113" t="s">
+        <v>459</v>
       </c>
     </row>
   </sheetData>
@@ -9239,308 +8542,42 @@
     <sortCondition ref="B2:B89"/>
   </sortState>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="E2:E21">
-    <cfRule type="beginsWith" dxfId="95" priority="85" operator="beginsWith" text="L">
+  <conditionalFormatting sqref="E2:E113">
+    <cfRule type="beginsWith" dxfId="11" priority="1" operator="beginsWith" text="L">
       <formula>LEFT(E2,LEN("L"))="L"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="94" priority="86" operator="beginsWith" text="K">
+    <cfRule type="beginsWith" dxfId="10" priority="2" operator="beginsWith" text="K">
       <formula>LEFT(E2,LEN("K"))="K"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="93" priority="87" operator="beginsWith" text="J">
+    <cfRule type="beginsWith" dxfId="9" priority="3" operator="beginsWith" text="J">
       <formula>LEFT(E2,LEN("J"))="J"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="92" priority="88" operator="beginsWith" text="I">
+    <cfRule type="beginsWith" dxfId="8" priority="4" operator="beginsWith" text="I">
       <formula>LEFT(E2,LEN("I"))="I"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="91" priority="89" operator="beginsWith" text="H">
+    <cfRule type="beginsWith" dxfId="7" priority="5" operator="beginsWith" text="H">
       <formula>LEFT(E2,LEN("H"))="H"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="90" priority="90" operator="beginsWith" text="G">
+    <cfRule type="beginsWith" dxfId="6" priority="6" operator="beginsWith" text="G">
       <formula>LEFT(E2,LEN("G"))="G"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="89" priority="91" operator="beginsWith" text="F">
+    <cfRule type="beginsWith" dxfId="5" priority="7" operator="beginsWith" text="F">
       <formula>LEFT(E2,LEN("F"))="F"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="88" priority="92" operator="beginsWith" text="E">
+    <cfRule type="beginsWith" dxfId="4" priority="8" operator="beginsWith" text="E">
       <formula>LEFT(E2,LEN("E"))="E"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="87" priority="93" operator="beginsWith" text="D">
+    <cfRule type="beginsWith" dxfId="3" priority="9" operator="beginsWith" text="D">
       <formula>LEFT(E2,LEN("D"))="D"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="86" priority="94" operator="beginsWith" text="C">
+    <cfRule type="beginsWith" dxfId="2" priority="10" operator="beginsWith" text="C">
       <formula>LEFT(E2,LEN("C"))="C"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="85" priority="95" operator="beginsWith" text="B">
+    <cfRule type="beginsWith" dxfId="1" priority="11" operator="beginsWith" text="B">
       <formula>LEFT(E2,LEN("B"))="B"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="84" priority="96" operator="beginsWith" text="A">
+    <cfRule type="beginsWith" dxfId="0" priority="12" operator="beginsWith" text="A">
       <formula>LEFT(E2,LEN("A"))="A"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E22:E76">
-    <cfRule type="beginsWith" dxfId="83" priority="73" operator="beginsWith" text="L">
-      <formula>LEFT(E22,LEN("L"))="L"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="82" priority="74" operator="beginsWith" text="K">
-      <formula>LEFT(E22,LEN("K"))="K"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="81" priority="75" operator="beginsWith" text="J">
-      <formula>LEFT(E22,LEN("J"))="J"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="80" priority="76" operator="beginsWith" text="I">
-      <formula>LEFT(E22,LEN("I"))="I"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="79" priority="77" operator="beginsWith" text="H">
-      <formula>LEFT(E22,LEN("H"))="H"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="78" priority="78" operator="beginsWith" text="G">
-      <formula>LEFT(E22,LEN("G"))="G"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="77" priority="79" operator="beginsWith" text="F">
-      <formula>LEFT(E22,LEN("F"))="F"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="76" priority="80" operator="beginsWith" text="E">
-      <formula>LEFT(E22,LEN("E"))="E"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="75" priority="81" operator="beginsWith" text="D">
-      <formula>LEFT(E22,LEN("D"))="D"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="74" priority="82" operator="beginsWith" text="C">
-      <formula>LEFT(E22,LEN("C"))="C"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="73" priority="83" operator="beginsWith" text="B">
-      <formula>LEFT(E22,LEN("B"))="B"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="72" priority="84" operator="beginsWith" text="A">
-      <formula>LEFT(E22,LEN("A"))="A"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E77:E94">
-    <cfRule type="beginsWith" dxfId="71" priority="61" operator="beginsWith" text="L">
-      <formula>LEFT(E77,LEN("L"))="L"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="70" priority="62" operator="beginsWith" text="K">
-      <formula>LEFT(E77,LEN("K"))="K"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="69" priority="63" operator="beginsWith" text="J">
-      <formula>LEFT(E77,LEN("J"))="J"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="68" priority="64" operator="beginsWith" text="I">
-      <formula>LEFT(E77,LEN("I"))="I"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="67" priority="65" operator="beginsWith" text="H">
-      <formula>LEFT(E77,LEN("H"))="H"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="66" priority="66" operator="beginsWith" text="G">
-      <formula>LEFT(E77,LEN("G"))="G"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="65" priority="67" operator="beginsWith" text="F">
-      <formula>LEFT(E77,LEN("F"))="F"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="64" priority="68" operator="beginsWith" text="E">
-      <formula>LEFT(E77,LEN("E"))="E"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="63" priority="69" operator="beginsWith" text="D">
-      <formula>LEFT(E77,LEN("D"))="D"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="62" priority="70" operator="beginsWith" text="C">
-      <formula>LEFT(E77,LEN("C"))="C"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="61" priority="71" operator="beginsWith" text="B">
-      <formula>LEFT(E77,LEN("B"))="B"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="60" priority="72" operator="beginsWith" text="A">
-      <formula>LEFT(E77,LEN("A"))="A"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E95">
-    <cfRule type="beginsWith" dxfId="59" priority="49" operator="beginsWith" text="L">
-      <formula>LEFT(E95,LEN("L"))="L"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="58" priority="50" operator="beginsWith" text="K">
-      <formula>LEFT(E95,LEN("K"))="K"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="57" priority="51" operator="beginsWith" text="J">
-      <formula>LEFT(E95,LEN("J"))="J"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="56" priority="52" operator="beginsWith" text="I">
-      <formula>LEFT(E95,LEN("I"))="I"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="55" priority="53" operator="beginsWith" text="H">
-      <formula>LEFT(E95,LEN("H"))="H"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="54" priority="54" operator="beginsWith" text="G">
-      <formula>LEFT(E95,LEN("G"))="G"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="53" priority="55" operator="beginsWith" text="F">
-      <formula>LEFT(E95,LEN("F"))="F"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="52" priority="56" operator="beginsWith" text="E">
-      <formula>LEFT(E95,LEN("E"))="E"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="51" priority="57" operator="beginsWith" text="D">
-      <formula>LEFT(E95,LEN("D"))="D"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="50" priority="58" operator="beginsWith" text="C">
-      <formula>LEFT(E95,LEN("C"))="C"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="49" priority="59" operator="beginsWith" text="B">
-      <formula>LEFT(E95,LEN("B"))="B"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="48" priority="60" operator="beginsWith" text="A">
-      <formula>LEFT(E95,LEN("A"))="A"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E96:E97">
-    <cfRule type="beginsWith" dxfId="47" priority="37" operator="beginsWith" text="L">
-      <formula>LEFT(E96,LEN("L"))="L"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="46" priority="38" operator="beginsWith" text="K">
-      <formula>LEFT(E96,LEN("K"))="K"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="45" priority="39" operator="beginsWith" text="J">
-      <formula>LEFT(E96,LEN("J"))="J"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="44" priority="40" operator="beginsWith" text="I">
-      <formula>LEFT(E96,LEN("I"))="I"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="43" priority="41" operator="beginsWith" text="H">
-      <formula>LEFT(E96,LEN("H"))="H"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="42" priority="42" operator="beginsWith" text="G">
-      <formula>LEFT(E96,LEN("G"))="G"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="41" priority="43" operator="beginsWith" text="F">
-      <formula>LEFT(E96,LEN("F"))="F"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="40" priority="44" operator="beginsWith" text="E">
-      <formula>LEFT(E96,LEN("E"))="E"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="39" priority="45" operator="beginsWith" text="D">
-      <formula>LEFT(E96,LEN("D"))="D"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="38" priority="46" operator="beginsWith" text="C">
-      <formula>LEFT(E96,LEN("C"))="C"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="37" priority="47" operator="beginsWith" text="B">
-      <formula>LEFT(E96,LEN("B"))="B"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="36" priority="48" operator="beginsWith" text="A">
-      <formula>LEFT(E96,LEN("A"))="A"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E98:E100">
-    <cfRule type="beginsWith" dxfId="35" priority="25" operator="beginsWith" text="L">
-      <formula>LEFT(E98,LEN("L"))="L"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="34" priority="26" operator="beginsWith" text="K">
-      <formula>LEFT(E98,LEN("K"))="K"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="33" priority="27" operator="beginsWith" text="J">
-      <formula>LEFT(E98,LEN("J"))="J"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="32" priority="28" operator="beginsWith" text="I">
-      <formula>LEFT(E98,LEN("I"))="I"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="31" priority="29" operator="beginsWith" text="H">
-      <formula>LEFT(E98,LEN("H"))="H"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="30" priority="30" operator="beginsWith" text="G">
-      <formula>LEFT(E98,LEN("G"))="G"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="29" priority="31" operator="beginsWith" text="F">
-      <formula>LEFT(E98,LEN("F"))="F"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="28" priority="32" operator="beginsWith" text="E">
-      <formula>LEFT(E98,LEN("E"))="E"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="27" priority="33" operator="beginsWith" text="D">
-      <formula>LEFT(E98,LEN("D"))="D"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="26" priority="34" operator="beginsWith" text="C">
-      <formula>LEFT(E98,LEN("C"))="C"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="25" priority="35" operator="beginsWith" text="B">
-      <formula>LEFT(E98,LEN("B"))="B"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="24" priority="36" operator="beginsWith" text="A">
-      <formula>LEFT(E98,LEN("A"))="A"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E106:E107">
-    <cfRule type="beginsWith" dxfId="23" priority="13" operator="beginsWith" text="L">
-      <formula>LEFT(E106,LEN("L"))="L"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="22" priority="14" operator="beginsWith" text="K">
-      <formula>LEFT(E106,LEN("K"))="K"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="21" priority="15" operator="beginsWith" text="J">
-      <formula>LEFT(E106,LEN("J"))="J"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="20" priority="16" operator="beginsWith" text="I">
-      <formula>LEFT(E106,LEN("I"))="I"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="19" priority="17" operator="beginsWith" text="H">
-      <formula>LEFT(E106,LEN("H"))="H"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="18" priority="18" operator="beginsWith" text="G">
-      <formula>LEFT(E106,LEN("G"))="G"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="17" priority="19" operator="beginsWith" text="F">
-      <formula>LEFT(E106,LEN("F"))="F"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="16" priority="20" operator="beginsWith" text="E">
-      <formula>LEFT(E106,LEN("E"))="E"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="15" priority="21" operator="beginsWith" text="D">
-      <formula>LEFT(E106,LEN("D"))="D"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="14" priority="22" operator="beginsWith" text="C">
-      <formula>LEFT(E106,LEN("C"))="C"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="13" priority="23" operator="beginsWith" text="B">
-      <formula>LEFT(E106,LEN("B"))="B"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="12" priority="24" operator="beginsWith" text="A">
-      <formula>LEFT(E106,LEN("A"))="A"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E101:E105">
-    <cfRule type="beginsWith" dxfId="11" priority="1" operator="beginsWith" text="L">
-      <formula>LEFT(E101,LEN("L"))="L"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="10" priority="2" operator="beginsWith" text="K">
-      <formula>LEFT(E101,LEN("K"))="K"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="9" priority="3" operator="beginsWith" text="J">
-      <formula>LEFT(E101,LEN("J"))="J"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="8" priority="4" operator="beginsWith" text="I">
-      <formula>LEFT(E101,LEN("I"))="I"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="7" priority="5" operator="beginsWith" text="H">
-      <formula>LEFT(E101,LEN("H"))="H"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="6" priority="6" operator="beginsWith" text="G">
-      <formula>LEFT(E101,LEN("G"))="G"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="5" priority="7" operator="beginsWith" text="F">
-      <formula>LEFT(E101,LEN("F"))="F"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="4" priority="8" operator="beginsWith" text="E">
-      <formula>LEFT(E101,LEN("E"))="E"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="3" priority="9" operator="beginsWith" text="D">
-      <formula>LEFT(E101,LEN("D"))="D"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="2" priority="10" operator="beginsWith" text="C">
-      <formula>LEFT(E101,LEN("C"))="C"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="1" priority="11" operator="beginsWith" text="B">
-      <formula>LEFT(E101,LEN("B"))="B"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="0" priority="12" operator="beginsWith" text="A">
-      <formula>LEFT(E101,LEN("A"))="A"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9570,7 +8607,7 @@
       <c r="A2" t="s">
         <v>329</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="35" t="s">
         <v>443</v>
       </c>
       <c r="C2" t="s">
@@ -9581,7 +8618,7 @@
       <c r="A3" t="s">
         <v>330</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="36" t="s">
         <v>444</v>
       </c>
       <c r="C3" t="s">
@@ -9592,7 +8629,7 @@
       <c r="A4" t="s">
         <v>331</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="37" t="s">
         <v>445</v>
       </c>
       <c r="C4" t="s">
@@ -9603,7 +8640,7 @@
       <c r="A5" t="s">
         <v>332</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="38" t="s">
         <v>446</v>
       </c>
       <c r="C5" t="s">
@@ -9614,7 +8651,7 @@
       <c r="A6" t="s">
         <v>333</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="39" t="s">
         <v>447</v>
       </c>
       <c r="C6" t="s">
@@ -9625,7 +8662,7 @@
       <c r="A7" t="s">
         <v>334</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="40" t="s">
         <v>448</v>
       </c>
       <c r="C7" t="s">
@@ -9636,7 +8673,7 @@
       <c r="A8" t="s">
         <v>335</v>
       </c>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="41" t="s">
         <v>449</v>
       </c>
       <c r="C8" t="s">
@@ -9647,7 +8684,7 @@
       <c r="A9" t="s">
         <v>336</v>
       </c>
-      <c r="B9" s="43" t="s">
+      <c r="B9" s="42" t="s">
         <v>450</v>
       </c>
       <c r="C9" t="s">
@@ -9658,7 +8695,7 @@
       <c r="A10" t="s">
         <v>337</v>
       </c>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="43" t="s">
         <v>451</v>
       </c>
       <c r="C10" t="s">
@@ -9669,7 +8706,7 @@
       <c r="A11" t="s">
         <v>338</v>
       </c>
-      <c r="B11" s="45" t="s">
+      <c r="B11" s="44" t="s">
         <v>452</v>
       </c>
       <c r="C11" t="s">
@@ -9680,7 +8717,7 @@
       <c r="A12" t="s">
         <v>339</v>
       </c>
-      <c r="B12" s="46" t="s">
+      <c r="B12" s="45" t="s">
         <v>453</v>
       </c>
       <c r="C12" t="s">
@@ -9691,7 +8728,7 @@
       <c r="A13" t="s">
         <v>340</v>
       </c>
-      <c r="B13" s="47" t="s">
+      <c r="B13" s="46" t="s">
         <v>341</v>
       </c>
       <c r="C13" t="s">

</xml_diff>